<commit_message>
Update ALNs and cluster names
</commit_message>
<xml_diff>
--- a/backend/cypress/fixtures/test_workbooks/additional-eins-workbook.xlsx
+++ b/backend/cypress/fixtures/test_workbooks/additional-eins-workbook.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lynnm\FAC\backend\schemas\output\excel\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7094EFA2-8248-40A1-8DA8-D2BEF673FFB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E1E15A-0312-4BA0-A17C-47C851FCF23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="8625" yWindow="-13815" windowWidth="21345" windowHeight="11490" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11370" yWindow="-14325" windowWidth="17280" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coversheet" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <definedName name="section_name">Coversheet!$B$3</definedName>
     <definedName name="version">Coversheet!$B$2</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -41,7 +41,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.1.7</t>
+    <t>1.1.8</t>
   </si>
   <si>
     <t>Section</t>

</xml_diff>

<commit_message>
Update ALN and clusters and add instruction line and update Cypress workbook fixtures April 2026
</commit_message>
<xml_diff>
--- a/backend/cypress/fixtures/test_workbooks/additional-eins-workbook.xlsx
+++ b/backend/cypress/fixtures/test_workbooks/additional-eins-workbook.xlsx
@@ -5,13 +5,13 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lynnm\FAC\backend\schemas\output\excel\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lynnm\FAC\backend\cypress\fixtures\test_workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E1E15A-0312-4BA0-A17C-47C851FCF23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7C8792-3016-421D-9051-24660C3DC2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="11370" yWindow="-14325" windowWidth="17280" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16008" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coversheet" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="additional_ein">Form!$A$2:$A$10000</definedName>
-    <definedName name="auditee_uei">Coversheet!$B$4</definedName>
+    <definedName name="auditee_uei">Coversheet!$B$5</definedName>
     <definedName name="section_name">Coversheet!$B$3</definedName>
     <definedName name="version">Coversheet!$B$2</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Federal Audit Clearinghouse
 fac.gov</t>
@@ -64,12 +64,18 @@
   <si>
     <t>987654321</t>
   </si>
+  <si>
+    <t>Instructions</t>
+  </si>
+  <si>
+    <t>SF-SAC Section 8: Additional EINs</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,6 +93,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -118,10 +132,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -137,8 +152,10 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -439,11 +456,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="48" customWidth="1"/>
-    <col min="3" max="16384" width="13" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="13" hidden="1" customWidth="1"/>
+    <col min="4" max="16384" width="13" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -472,19 +490,30 @@
     </row>
     <row r="4" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
   <dataValidations count="1">
-    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" errorTitle="Must be length of 12" error="Expecting something with 12 characters" sqref="B4" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" errorTitle="Must be length of 12" error="Expecting something with 12 characters" sqref="B5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>12</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" display="https://www.fac.gov/audit-resources/sf-sac/additional-eins-workbook/" xr:uid="{035FE3FE-325C-4EC5-974C-18FC970E9513}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -492,10 +521,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A10000"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="16384" width="13" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="13" hidden="1" customWidth="1"/>
+    <col min="3" max="16384" width="13" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="48" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update workbooks to fix missing trailing zeroes and to add instruction line (#5531)
* Update README.md

changes to Sam.gov search interface; added a step for action after zeroes get dropped by Excel

* Update ALN and clusters and add instruction line and update Cypress workbook fixtures April 2026

---------

Co-authored-by: Phil Dominguez <142051477+phildominguez-gsa@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/backend/cypress/fixtures/test_workbooks/additional-eins-workbook.xlsx
+++ b/backend/cypress/fixtures/test_workbooks/additional-eins-workbook.xlsx
@@ -5,13 +5,13 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lynnm\FAC\backend\schemas\output\excel\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lynnm\FAC\backend\cypress\fixtures\test_workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E1E15A-0312-4BA0-A17C-47C851FCF23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7C8792-3016-421D-9051-24660C3DC2B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="11370" yWindow="-14325" windowWidth="17280" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16008" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coversheet" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="additional_ein">Form!$A$2:$A$10000</definedName>
-    <definedName name="auditee_uei">Coversheet!$B$4</definedName>
+    <definedName name="auditee_uei">Coversheet!$B$5</definedName>
     <definedName name="section_name">Coversheet!$B$3</definedName>
     <definedName name="version">Coversheet!$B$2</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Federal Audit Clearinghouse
 fac.gov</t>
@@ -64,12 +64,18 @@
   <si>
     <t>987654321</t>
   </si>
+  <si>
+    <t>Instructions</t>
+  </si>
+  <si>
+    <t>SF-SAC Section 8: Additional EINs</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,6 +93,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -118,10 +132,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -137,8 +152,10 @@
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -439,11 +456,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="48" customWidth="1"/>
-    <col min="3" max="16384" width="13" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="13" hidden="1" customWidth="1"/>
+    <col min="4" max="16384" width="13" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -472,19 +490,30 @@
     </row>
     <row r="4" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
   <dataValidations count="1">
-    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" errorTitle="Must be length of 12" error="Expecting something with 12 characters" sqref="B4" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="textLength" operator="equal" allowBlank="1" showErrorMessage="1" errorTitle="Must be length of 12" error="Expecting something with 12 characters" sqref="B5" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>12</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" display="https://www.fac.gov/audit-resources/sf-sac/additional-eins-workbook/" xr:uid="{035FE3FE-325C-4EC5-974C-18FC970E9513}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -492,10 +521,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A10000"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="16384" width="13" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="13" hidden="1" customWidth="1"/>
+    <col min="3" max="16384" width="13" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="48" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>